<commit_message>
Automatycznie wygenerowano nowe dane o
</commit_message>
<xml_diff>
--- a/dane.xlsx
+++ b/dane.xlsx
@@ -3759,7 +3759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G491"/>
+  <dimension ref="A1:G501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16047,6 +16047,256 @@
       </c>
       <c r="G491" t="n">
         <v>400</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="n">
+        <v>491</v>
+      </c>
+      <c r="B492" s="2" t="n">
+        <v>46068</v>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>Zwrot</t>
+        </is>
+      </c>
+      <c r="D492" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E492" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F492" t="n">
+        <v>1</v>
+      </c>
+      <c r="G492" t="n">
+        <v>2397</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="n">
+        <v>492</v>
+      </c>
+      <c r="B493" s="2" t="n">
+        <v>46072</v>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Wysłane</t>
+        </is>
+      </c>
+      <c r="D493" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="E493" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F493" t="n">
+        <v>4</v>
+      </c>
+      <c r="G493" t="n">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="n">
+        <v>493</v>
+      </c>
+      <c r="B494" s="2" t="n">
+        <v>46063</v>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Dostarczone</t>
+        </is>
+      </c>
+      <c r="D494" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E494" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F494" t="n">
+        <v>2</v>
+      </c>
+      <c r="G494" t="n">
+        <v>1953</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="n">
+        <v>494</v>
+      </c>
+      <c r="B495" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Nowe</t>
+        </is>
+      </c>
+      <c r="D495" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E495" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F495" t="n">
+        <v>3</v>
+      </c>
+      <c r="G495" t="n">
+        <v>1805</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="n">
+        <v>495</v>
+      </c>
+      <c r="B496" s="2" t="n">
+        <v>46075</v>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Wysłane</t>
+        </is>
+      </c>
+      <c r="D496" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="E496" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F496" t="n">
+        <v>3</v>
+      </c>
+      <c r="G496" t="n">
+        <v>2678</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="n">
+        <v>496</v>
+      </c>
+      <c r="B497" s="2" t="n">
+        <v>46071</v>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Zwrot</t>
+        </is>
+      </c>
+      <c r="D497" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E497" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F497" t="n">
+        <v>3</v>
+      </c>
+      <c r="G497" t="n">
+        <v>2586</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="n">
+        <v>497</v>
+      </c>
+      <c r="B498" s="2" t="n">
+        <v>46070</v>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Nowe</t>
+        </is>
+      </c>
+      <c r="D498" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="E498" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F498" t="n">
+        <v>2</v>
+      </c>
+      <c r="G498" t="n">
+        <v>2745</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="n">
+        <v>498</v>
+      </c>
+      <c r="B499" s="2" t="n">
+        <v>46080</v>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Nowe</t>
+        </is>
+      </c>
+      <c r="D499" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="E499" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F499" t="n">
+        <v>3</v>
+      </c>
+      <c r="G499" t="n">
+        <v>582</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="n">
+        <v>499</v>
+      </c>
+      <c r="B500" s="2" t="n">
+        <v>46077</v>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Nowe</t>
+        </is>
+      </c>
+      <c r="D500" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E500" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F500" t="n">
+        <v>1</v>
+      </c>
+      <c r="G500" t="n">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="n">
+        <v>500</v>
+      </c>
+      <c r="B501" s="2" t="n">
+        <v>46073</v>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Zwrot</t>
+        </is>
+      </c>
+      <c r="D501" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="E501" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F501" t="n">
+        <v>2</v>
+      </c>
+      <c r="G501" t="n">
+        <v>1062</v>
       </c>
     </row>
   </sheetData>
@@ -16060,7 +16310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3014"/>
+  <dimension ref="A1:E3072"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -59006,6 +59256,992 @@
       </c>
       <c r="E3014" t="n">
         <v>490</v>
+      </c>
+    </row>
+    <row r="3015">
+      <c r="A3015" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3015" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3015" t="n">
+        <v>52</v>
+      </c>
+      <c r="D3015" t="n">
+        <v>48</v>
+      </c>
+      <c r="E3015" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3016">
+      <c r="A3016" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3016" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3016" t="n">
+        <v>70</v>
+      </c>
+      <c r="D3016" t="n">
+        <v>86</v>
+      </c>
+      <c r="E3016" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3017">
+      <c r="A3017" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3017" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3017" t="n">
+        <v>62</v>
+      </c>
+      <c r="D3017" t="n">
+        <v>80</v>
+      </c>
+      <c r="E3017" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3018">
+      <c r="A3018" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3018" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3018" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3018" t="n">
+        <v>47</v>
+      </c>
+      <c r="E3018" t="n">
+        <v>491</v>
+      </c>
+    </row>
+    <row r="3019">
+      <c r="A3019" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3019" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3019" t="n">
+        <v>79</v>
+      </c>
+      <c r="D3019" t="n">
+        <v>15</v>
+      </c>
+      <c r="E3019" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3020">
+      <c r="A3020" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3020" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3020" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3020" t="n">
+        <v>63</v>
+      </c>
+      <c r="E3020" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3021">
+      <c r="A3021" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3021" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3021" t="n">
+        <v>42</v>
+      </c>
+      <c r="D3021" t="n">
+        <v>43</v>
+      </c>
+      <c r="E3021" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3022">
+      <c r="A3022" t="n">
+        <v>7</v>
+      </c>
+      <c r="B3022" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3022" t="n">
+        <v>86</v>
+      </c>
+      <c r="D3022" t="n">
+        <v>75</v>
+      </c>
+      <c r="E3022" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3023">
+      <c r="A3023" t="n">
+        <v>8</v>
+      </c>
+      <c r="B3023" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3023" t="n">
+        <v>38</v>
+      </c>
+      <c r="D3023" t="n">
+        <v>89</v>
+      </c>
+      <c r="E3023" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3024">
+      <c r="A3024" t="n">
+        <v>9</v>
+      </c>
+      <c r="B3024" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3024" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3024" t="n">
+        <v>24</v>
+      </c>
+      <c r="E3024" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3025">
+      <c r="A3025" t="n">
+        <v>10</v>
+      </c>
+      <c r="B3025" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3025" t="n">
+        <v>65</v>
+      </c>
+      <c r="D3025" t="n">
+        <v>11</v>
+      </c>
+      <c r="E3025" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3026">
+      <c r="A3026" t="n">
+        <v>11</v>
+      </c>
+      <c r="B3026" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3026" t="n">
+        <v>68</v>
+      </c>
+      <c r="D3026" t="n">
+        <v>81</v>
+      </c>
+      <c r="E3026" t="n">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="3027">
+      <c r="A3027" t="n">
+        <v>12</v>
+      </c>
+      <c r="B3027" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3027" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3027" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3027" t="n">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="3028">
+      <c r="A3028" t="n">
+        <v>13</v>
+      </c>
+      <c r="B3028" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3028" t="n">
+        <v>91</v>
+      </c>
+      <c r="D3028" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3028" t="n">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="3029">
+      <c r="A3029" t="n">
+        <v>14</v>
+      </c>
+      <c r="B3029" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3029" t="n">
+        <v>64</v>
+      </c>
+      <c r="D3029" t="n">
+        <v>60</v>
+      </c>
+      <c r="E3029" t="n">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="3030">
+      <c r="A3030" t="n">
+        <v>15</v>
+      </c>
+      <c r="B3030" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3030" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3030" t="n">
+        <v>93</v>
+      </c>
+      <c r="E3030" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3031">
+      <c r="A3031" t="n">
+        <v>16</v>
+      </c>
+      <c r="B3031" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3031" t="n">
+        <v>66</v>
+      </c>
+      <c r="D3031" t="n">
+        <v>82</v>
+      </c>
+      <c r="E3031" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3032">
+      <c r="A3032" t="n">
+        <v>17</v>
+      </c>
+      <c r="B3032" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3032" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3032" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3032" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3033">
+      <c r="A3033" t="n">
+        <v>18</v>
+      </c>
+      <c r="B3033" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3033" t="n">
+        <v>57</v>
+      </c>
+      <c r="D3033" t="n">
+        <v>99</v>
+      </c>
+      <c r="E3033" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3034">
+      <c r="A3034" t="n">
+        <v>19</v>
+      </c>
+      <c r="B3034" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3034" t="n">
+        <v>60</v>
+      </c>
+      <c r="D3034" t="n">
+        <v>39</v>
+      </c>
+      <c r="E3034" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3035">
+      <c r="A3035" t="n">
+        <v>20</v>
+      </c>
+      <c r="B3035" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3035" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3035" t="n">
+        <v>61</v>
+      </c>
+      <c r="E3035" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3036">
+      <c r="A3036" t="n">
+        <v>21</v>
+      </c>
+      <c r="B3036" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3036" t="n">
+        <v>22</v>
+      </c>
+      <c r="D3036" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3036" t="n">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="3037">
+      <c r="A3037" t="n">
+        <v>22</v>
+      </c>
+      <c r="B3037" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3037" t="n">
+        <v>71</v>
+      </c>
+      <c r="D3037" t="n">
+        <v>41</v>
+      </c>
+      <c r="E3037" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3038">
+      <c r="A3038" t="n">
+        <v>23</v>
+      </c>
+      <c r="B3038" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3038" t="n">
+        <v>77</v>
+      </c>
+      <c r="D3038" t="n">
+        <v>93</v>
+      </c>
+      <c r="E3038" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3039">
+      <c r="A3039" t="n">
+        <v>24</v>
+      </c>
+      <c r="B3039" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3039" t="n">
+        <v>98</v>
+      </c>
+      <c r="D3039" t="n">
+        <v>27</v>
+      </c>
+      <c r="E3039" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3040">
+      <c r="A3040" t="n">
+        <v>25</v>
+      </c>
+      <c r="B3040" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3040" t="n">
+        <v>87</v>
+      </c>
+      <c r="D3040" t="n">
+        <v>46</v>
+      </c>
+      <c r="E3040" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3041">
+      <c r="A3041" t="n">
+        <v>26</v>
+      </c>
+      <c r="B3041" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3041" t="n">
+        <v>53</v>
+      </c>
+      <c r="D3041" t="n">
+        <v>67</v>
+      </c>
+      <c r="E3041" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3042">
+      <c r="A3042" t="n">
+        <v>27</v>
+      </c>
+      <c r="B3042" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3042" t="n">
+        <v>95</v>
+      </c>
+      <c r="D3042" t="n">
+        <v>26</v>
+      </c>
+      <c r="E3042" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3043">
+      <c r="A3043" t="n">
+        <v>28</v>
+      </c>
+      <c r="B3043" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3043" t="n">
+        <v>52</v>
+      </c>
+      <c r="D3043" t="n">
+        <v>75</v>
+      </c>
+      <c r="E3043" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="3044">
+      <c r="A3044" t="n">
+        <v>29</v>
+      </c>
+      <c r="B3044" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3044" t="n">
+        <v>95</v>
+      </c>
+      <c r="D3044" t="n">
+        <v>71</v>
+      </c>
+      <c r="E3044" t="n">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="3045">
+      <c r="A3045" t="n">
+        <v>30</v>
+      </c>
+      <c r="B3045" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3045" t="n">
+        <v>40</v>
+      </c>
+      <c r="D3045" t="n">
+        <v>91</v>
+      </c>
+      <c r="E3045" t="n">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="3046">
+      <c r="A3046" t="n">
+        <v>31</v>
+      </c>
+      <c r="B3046" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3046" t="n">
+        <v>47</v>
+      </c>
+      <c r="D3046" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3046" t="n">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="3047">
+      <c r="A3047" t="n">
+        <v>32</v>
+      </c>
+      <c r="B3047" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3047" t="n">
+        <v>12</v>
+      </c>
+      <c r="D3047" t="n">
+        <v>61</v>
+      </c>
+      <c r="E3047" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="3048">
+      <c r="A3048" t="n">
+        <v>33</v>
+      </c>
+      <c r="B3048" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3048" t="n">
+        <v>78</v>
+      </c>
+      <c r="D3048" t="n">
+        <v>83</v>
+      </c>
+      <c r="E3048" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="3049">
+      <c r="A3049" t="n">
+        <v>34</v>
+      </c>
+      <c r="B3049" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3049" t="n">
+        <v>36</v>
+      </c>
+      <c r="D3049" t="n">
+        <v>27</v>
+      </c>
+      <c r="E3049" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="3050">
+      <c r="A3050" t="n">
+        <v>35</v>
+      </c>
+      <c r="B3050" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3050" t="n">
+        <v>31</v>
+      </c>
+      <c r="D3050" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3050" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="3051">
+      <c r="A3051" t="n">
+        <v>36</v>
+      </c>
+      <c r="B3051" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3051" t="n">
+        <v>71</v>
+      </c>
+      <c r="D3051" t="n">
+        <v>96</v>
+      </c>
+      <c r="E3051" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3052">
+      <c r="A3052" t="n">
+        <v>37</v>
+      </c>
+      <c r="B3052" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3052" t="n">
+        <v>59</v>
+      </c>
+      <c r="D3052" t="n">
+        <v>79</v>
+      </c>
+      <c r="E3052" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3053">
+      <c r="A3053" t="n">
+        <v>38</v>
+      </c>
+      <c r="B3053" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3053" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3053" t="n">
+        <v>26</v>
+      </c>
+      <c r="E3053" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3054">
+      <c r="A3054" t="n">
+        <v>39</v>
+      </c>
+      <c r="B3054" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3054" t="n">
+        <v>71</v>
+      </c>
+      <c r="D3054" t="n">
+        <v>69</v>
+      </c>
+      <c r="E3054" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3055">
+      <c r="A3055" t="n">
+        <v>40</v>
+      </c>
+      <c r="B3055" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3055" t="n">
+        <v>42</v>
+      </c>
+      <c r="D3055" t="n">
+        <v>39</v>
+      </c>
+      <c r="E3055" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3056">
+      <c r="A3056" t="n">
+        <v>41</v>
+      </c>
+      <c r="B3056" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3056" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3056" t="n">
+        <v>53</v>
+      </c>
+      <c r="E3056" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3057">
+      <c r="A3057" t="n">
+        <v>42</v>
+      </c>
+      <c r="B3057" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3057" t="n">
+        <v>100</v>
+      </c>
+      <c r="D3057" t="n">
+        <v>10</v>
+      </c>
+      <c r="E3057" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3058">
+      <c r="A3058" t="n">
+        <v>43</v>
+      </c>
+      <c r="B3058" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3058" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3058" t="n">
+        <v>90</v>
+      </c>
+      <c r="E3058" t="n">
+        <v>498</v>
+      </c>
+    </row>
+    <row r="3059">
+      <c r="A3059" t="n">
+        <v>44</v>
+      </c>
+      <c r="B3059" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3059" t="n">
+        <v>75</v>
+      </c>
+      <c r="D3059" t="n">
+        <v>66</v>
+      </c>
+      <c r="E3059" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="3060">
+      <c r="A3060" t="n">
+        <v>45</v>
+      </c>
+      <c r="B3060" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3060" t="n">
+        <v>97</v>
+      </c>
+      <c r="D3060" t="n">
+        <v>42</v>
+      </c>
+      <c r="E3060" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="3061">
+      <c r="A3061" t="n">
+        <v>46</v>
+      </c>
+      <c r="B3061" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3061" t="n">
+        <v>96</v>
+      </c>
+      <c r="D3061" t="n">
+        <v>25</v>
+      </c>
+      <c r="E3061" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="3062">
+      <c r="A3062" t="n">
+        <v>47</v>
+      </c>
+      <c r="B3062" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3062" t="n">
+        <v>50</v>
+      </c>
+      <c r="D3062" t="n">
+        <v>84</v>
+      </c>
+      <c r="E3062" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="3063">
+      <c r="A3063" t="n">
+        <v>48</v>
+      </c>
+      <c r="B3063" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3063" t="n">
+        <v>46</v>
+      </c>
+      <c r="D3063" t="n">
+        <v>40</v>
+      </c>
+      <c r="E3063" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="3064">
+      <c r="A3064" t="n">
+        <v>49</v>
+      </c>
+      <c r="B3064" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3064" t="n">
+        <v>90</v>
+      </c>
+      <c r="D3064" t="n">
+        <v>82</v>
+      </c>
+      <c r="E3064" t="n">
+        <v>499</v>
+      </c>
+    </row>
+    <row r="3065">
+      <c r="A3065" t="n">
+        <v>50</v>
+      </c>
+      <c r="B3065" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3065" t="n">
+        <v>84</v>
+      </c>
+      <c r="D3065" t="n">
+        <v>98</v>
+      </c>
+      <c r="E3065" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3066">
+      <c r="A3066" t="n">
+        <v>51</v>
+      </c>
+      <c r="B3066" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3066" t="n">
+        <v>27</v>
+      </c>
+      <c r="D3066" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3066" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3067">
+      <c r="A3067" t="n">
+        <v>52</v>
+      </c>
+      <c r="B3067" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3067" t="n">
+        <v>70</v>
+      </c>
+      <c r="D3067" t="n">
+        <v>85</v>
+      </c>
+      <c r="E3067" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3068">
+      <c r="A3068" t="n">
+        <v>53</v>
+      </c>
+      <c r="B3068" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3068" t="n">
+        <v>66</v>
+      </c>
+      <c r="D3068" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3068" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3069">
+      <c r="A3069" t="n">
+        <v>54</v>
+      </c>
+      <c r="B3069" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3069" t="n">
+        <v>82</v>
+      </c>
+      <c r="D3069" t="n">
+        <v>57</v>
+      </c>
+      <c r="E3069" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3070">
+      <c r="A3070" t="n">
+        <v>55</v>
+      </c>
+      <c r="B3070" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3070" t="n">
+        <v>52</v>
+      </c>
+      <c r="D3070" t="n">
+        <v>89</v>
+      </c>
+      <c r="E3070" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3071">
+      <c r="A3071" t="n">
+        <v>56</v>
+      </c>
+      <c r="B3071" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3071" t="n">
+        <v>76</v>
+      </c>
+      <c r="D3071" t="n">
+        <v>91</v>
+      </c>
+      <c r="E3071" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="3072">
+      <c r="A3072" t="n">
+        <v>57</v>
+      </c>
+      <c r="B3072" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3072" t="n">
+        <v>85</v>
+      </c>
+      <c r="D3072" t="n">
+        <v>93</v>
+      </c>
+      <c r="E3072" t="n">
+        <v>500</v>
       </c>
     </row>
   </sheetData>
@@ -59019,7 +60255,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F213"/>
+  <dimension ref="A1:F216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64964,30 +66200,114 @@
     </row>
     <row r="213">
       <c r="A213" t="n">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Glow Opole</t>
+          <t>Vita Pro</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>9125752553</t>
+          <t>0039863389</t>
         </is>
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>Elbląg</t>
+          <t>Radom</t>
         </is>
       </c>
       <c r="E213" t="inlineStr">
         <is>
+          <t>Sklep internetowy z suplementami</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="n">
+        <v>218</v>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Care Pure </t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>9163561334</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Zabrze</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
           <t>Medycyna estetyczna / klinika urody</t>
         </is>
       </c>
-      <c r="F213" t="n">
-        <v>2</v>
+      <c r="F214" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="n">
+        <v>219</v>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Well Power Zabrze</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>8678424220</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Koło</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Medycyna estetyczna / klinika urody</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="n">
+        <v>220</v>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Energy Power Radom</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>4609605632</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Opole</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Siłownia / klub sportowy</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Automatycznie wygenerowano nowe dane
</commit_message>
<xml_diff>
--- a/dane.xlsx
+++ b/dane.xlsx
@@ -3759,7 +3759,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G551"/>
+  <dimension ref="A1:G561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17547,6 +17547,256 @@
       </c>
       <c r="G551" t="n">
         <v>1408</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="n">
+        <v>551</v>
+      </c>
+      <c r="B552" s="2" t="n">
+        <v>46064</v>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Wysłane</t>
+        </is>
+      </c>
+      <c r="D552" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E552" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F552" t="n">
+        <v>3</v>
+      </c>
+      <c r="G552" t="n">
+        <v>1101</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="n">
+        <v>552</v>
+      </c>
+      <c r="B553" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Zwrot</t>
+        </is>
+      </c>
+      <c r="D553" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="E553" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F553" t="n">
+        <v>3</v>
+      </c>
+      <c r="G553" t="n">
+        <v>2346</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="n">
+        <v>553</v>
+      </c>
+      <c r="B554" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Nowe</t>
+        </is>
+      </c>
+      <c r="D554" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="E554" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F554" t="n">
+        <v>4</v>
+      </c>
+      <c r="G554" t="n">
+        <v>2514</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="n">
+        <v>554</v>
+      </c>
+      <c r="B555" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Zwrot</t>
+        </is>
+      </c>
+      <c r="D555" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E555" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F555" t="n">
+        <v>3</v>
+      </c>
+      <c r="G555" t="n">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="n">
+        <v>555</v>
+      </c>
+      <c r="B556" s="2" t="n">
+        <v>46078</v>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Nowe</t>
+        </is>
+      </c>
+      <c r="D556" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="E556" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F556" t="n">
+        <v>2</v>
+      </c>
+      <c r="G556" t="n">
+        <v>3321</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="n">
+        <v>556</v>
+      </c>
+      <c r="B557" s="2" t="n">
+        <v>46082</v>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Zwrot</t>
+        </is>
+      </c>
+      <c r="D557" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="E557" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F557" t="n">
+        <v>3</v>
+      </c>
+      <c r="G557" t="n">
+        <v>2860</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="n">
+        <v>557</v>
+      </c>
+      <c r="B558" s="2" t="n">
+        <v>46064</v>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Dostarczone</t>
+        </is>
+      </c>
+      <c r="D558" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="E558" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F558" t="n">
+        <v>1</v>
+      </c>
+      <c r="G558" t="n">
+        <v>1628</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="n">
+        <v>558</v>
+      </c>
+      <c r="B559" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Wysłane</t>
+        </is>
+      </c>
+      <c r="D559" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E559" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F559" t="n">
+        <v>1</v>
+      </c>
+      <c r="G559" t="n">
+        <v>2467</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="n">
+        <v>559</v>
+      </c>
+      <c r="B560" s="2" t="n">
+        <v>46083</v>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Dostarczone</t>
+        </is>
+      </c>
+      <c r="D560" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E560" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F560" t="n">
+        <v>1</v>
+      </c>
+      <c r="G560" t="n">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="n">
+        <v>560</v>
+      </c>
+      <c r="B561" s="2" t="n">
+        <v>46076</v>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Zwrot</t>
+        </is>
+      </c>
+      <c r="D561" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="E561" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F561" t="n">
+        <v>2</v>
+      </c>
+      <c r="G561" t="n">
+        <v>920</v>
       </c>
     </row>
   </sheetData>
@@ -17560,7 +17810,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3375"/>
+  <dimension ref="A1:E3426"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -66643,6 +66893,873 @@
       </c>
       <c r="E3375" t="n">
         <v>550</v>
+      </c>
+    </row>
+    <row r="3376">
+      <c r="A3376" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3376" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3376" t="n">
+        <v>82</v>
+      </c>
+      <c r="D3376" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3376" t="n">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="3377">
+      <c r="A3377" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3377" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3377" t="n">
+        <v>77</v>
+      </c>
+      <c r="D3377" t="n">
+        <v>58</v>
+      </c>
+      <c r="E3377" t="n">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="3378">
+      <c r="A3378" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3378" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3378" t="n">
+        <v>55</v>
+      </c>
+      <c r="D3378" t="n">
+        <v>39</v>
+      </c>
+      <c r="E3378" t="n">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="3379">
+      <c r="A3379" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3379" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3379" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3379" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3379" t="n">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="3380">
+      <c r="A3380" t="n">
+        <v>4</v>
+      </c>
+      <c r="B3380" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3380" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3380" t="n">
+        <v>47</v>
+      </c>
+      <c r="E3380" t="n">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="3381">
+      <c r="A3381" t="n">
+        <v>5</v>
+      </c>
+      <c r="B3381" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3381" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3381" t="n">
+        <v>97</v>
+      </c>
+      <c r="E3381" t="n">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="3382">
+      <c r="A3382" t="n">
+        <v>6</v>
+      </c>
+      <c r="B3382" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3382" t="n">
+        <v>57</v>
+      </c>
+      <c r="D3382" t="n">
+        <v>85</v>
+      </c>
+      <c r="E3382" t="n">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="3383">
+      <c r="A3383" t="n">
+        <v>7</v>
+      </c>
+      <c r="B3383" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3383" t="n">
+        <v>66</v>
+      </c>
+      <c r="D3383" t="n">
+        <v>39</v>
+      </c>
+      <c r="E3383" t="n">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="3384">
+      <c r="A3384" t="n">
+        <v>8</v>
+      </c>
+      <c r="B3384" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3384" t="n">
+        <v>21</v>
+      </c>
+      <c r="D3384" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3384" t="n">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="3385">
+      <c r="A3385" t="n">
+        <v>9</v>
+      </c>
+      <c r="B3385" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3385" t="n">
+        <v>23</v>
+      </c>
+      <c r="D3385" t="n">
+        <v>45</v>
+      </c>
+      <c r="E3385" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3386">
+      <c r="A3386" t="n">
+        <v>10</v>
+      </c>
+      <c r="B3386" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3386" t="n">
+        <v>60</v>
+      </c>
+      <c r="D3386" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3386" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3387">
+      <c r="A3387" t="n">
+        <v>11</v>
+      </c>
+      <c r="B3387" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3387" t="n">
+        <v>93</v>
+      </c>
+      <c r="D3387" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3387" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3388">
+      <c r="A3388" t="n">
+        <v>12</v>
+      </c>
+      <c r="B3388" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3388" t="n">
+        <v>5</v>
+      </c>
+      <c r="D3388" t="n">
+        <v>18</v>
+      </c>
+      <c r="E3388" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3389">
+      <c r="A3389" t="n">
+        <v>13</v>
+      </c>
+      <c r="B3389" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3389" t="n">
+        <v>37</v>
+      </c>
+      <c r="D3389" t="n">
+        <v>16</v>
+      </c>
+      <c r="E3389" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3390">
+      <c r="A3390" t="n">
+        <v>14</v>
+      </c>
+      <c r="B3390" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3390" t="n">
+        <v>17</v>
+      </c>
+      <c r="D3390" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3390" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3391">
+      <c r="A3391" t="n">
+        <v>15</v>
+      </c>
+      <c r="B3391" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3391" t="n">
+        <v>98</v>
+      </c>
+      <c r="D3391" t="n">
+        <v>92</v>
+      </c>
+      <c r="E3391" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3392">
+      <c r="A3392" t="n">
+        <v>16</v>
+      </c>
+      <c r="B3392" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3392" t="n">
+        <v>14</v>
+      </c>
+      <c r="D3392" t="n">
+        <v>86</v>
+      </c>
+      <c r="E3392" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3393">
+      <c r="A3393" t="n">
+        <v>17</v>
+      </c>
+      <c r="B3393" t="n">
+        <v>9</v>
+      </c>
+      <c r="C3393" t="n">
+        <v>91</v>
+      </c>
+      <c r="D3393" t="n">
+        <v>27</v>
+      </c>
+      <c r="E3393" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3394">
+      <c r="A3394" t="n">
+        <v>18</v>
+      </c>
+      <c r="B3394" t="n">
+        <v>10</v>
+      </c>
+      <c r="C3394" t="n">
+        <v>98</v>
+      </c>
+      <c r="D3394" t="n">
+        <v>47</v>
+      </c>
+      <c r="E3394" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="3395">
+      <c r="A3395" t="n">
+        <v>19</v>
+      </c>
+      <c r="B3395" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3395" t="n">
+        <v>49</v>
+      </c>
+      <c r="D3395" t="n">
+        <v>19</v>
+      </c>
+      <c r="E3395" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="3396">
+      <c r="A3396" t="n">
+        <v>20</v>
+      </c>
+      <c r="B3396" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3396" t="n">
+        <v>65</v>
+      </c>
+      <c r="D3396" t="n">
+        <v>59</v>
+      </c>
+      <c r="E3396" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="3397">
+      <c r="A3397" t="n">
+        <v>21</v>
+      </c>
+      <c r="B3397" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3397" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3397" t="n">
+        <v>66</v>
+      </c>
+      <c r="E3397" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="3398">
+      <c r="A3398" t="n">
+        <v>22</v>
+      </c>
+      <c r="B3398" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3398" t="n">
+        <v>61</v>
+      </c>
+      <c r="D3398" t="n">
+        <v>50</v>
+      </c>
+      <c r="E3398" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="3399">
+      <c r="A3399" t="n">
+        <v>23</v>
+      </c>
+      <c r="B3399" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3399" t="n">
+        <v>67</v>
+      </c>
+      <c r="D3399" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3399" t="n">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="3400">
+      <c r="A3400" t="n">
+        <v>24</v>
+      </c>
+      <c r="B3400" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3400" t="n">
+        <v>96</v>
+      </c>
+      <c r="D3400" t="n">
+        <v>24</v>
+      </c>
+      <c r="E3400" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="3401">
+      <c r="A3401" t="n">
+        <v>25</v>
+      </c>
+      <c r="B3401" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3401" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3401" t="n">
+        <v>97</v>
+      </c>
+      <c r="E3401" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="3402">
+      <c r="A3402" t="n">
+        <v>26</v>
+      </c>
+      <c r="B3402" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3402" t="n">
+        <v>23</v>
+      </c>
+      <c r="D3402" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3402" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="3403">
+      <c r="A3403" t="n">
+        <v>27</v>
+      </c>
+      <c r="B3403" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3403" t="n">
+        <v>93</v>
+      </c>
+      <c r="D3403" t="n">
+        <v>23</v>
+      </c>
+      <c r="E3403" t="n">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="3404">
+      <c r="A3404" t="n">
+        <v>28</v>
+      </c>
+      <c r="B3404" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3404" t="n">
+        <v>59</v>
+      </c>
+      <c r="D3404" t="n">
+        <v>31</v>
+      </c>
+      <c r="E3404" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3405">
+      <c r="A3405" t="n">
+        <v>29</v>
+      </c>
+      <c r="B3405" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3405" t="n">
+        <v>16</v>
+      </c>
+      <c r="D3405" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3405" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3406">
+      <c r="A3406" t="n">
+        <v>30</v>
+      </c>
+      <c r="B3406" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3406" t="n">
+        <v>46</v>
+      </c>
+      <c r="D3406" t="n">
+        <v>99</v>
+      </c>
+      <c r="E3406" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3407">
+      <c r="A3407" t="n">
+        <v>31</v>
+      </c>
+      <c r="B3407" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3407" t="n">
+        <v>42</v>
+      </c>
+      <c r="D3407" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3407" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3408">
+      <c r="A3408" t="n">
+        <v>32</v>
+      </c>
+      <c r="B3408" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3408" t="n">
+        <v>25</v>
+      </c>
+      <c r="D3408" t="n">
+        <v>34</v>
+      </c>
+      <c r="E3408" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3409">
+      <c r="A3409" t="n">
+        <v>33</v>
+      </c>
+      <c r="B3409" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3409" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3409" t="n">
+        <v>14</v>
+      </c>
+      <c r="E3409" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3410">
+      <c r="A3410" t="n">
+        <v>34</v>
+      </c>
+      <c r="B3410" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3410" t="n">
+        <v>11</v>
+      </c>
+      <c r="D3410" t="n">
+        <v>85</v>
+      </c>
+      <c r="E3410" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3411">
+      <c r="A3411" t="n">
+        <v>35</v>
+      </c>
+      <c r="B3411" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3411" t="n">
+        <v>18</v>
+      </c>
+      <c r="D3411" t="n">
+        <v>36</v>
+      </c>
+      <c r="E3411" t="n">
+        <v>557</v>
+      </c>
+    </row>
+    <row r="3412">
+      <c r="A3412" t="n">
+        <v>36</v>
+      </c>
+      <c r="B3412" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3412" t="n">
+        <v>86</v>
+      </c>
+      <c r="D3412" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3412" t="n">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="3413">
+      <c r="A3413" t="n">
+        <v>37</v>
+      </c>
+      <c r="B3413" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3413" t="n">
+        <v>54</v>
+      </c>
+      <c r="D3413" t="n">
+        <v>16</v>
+      </c>
+      <c r="E3413" t="n">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="3414">
+      <c r="A3414" t="n">
+        <v>38</v>
+      </c>
+      <c r="B3414" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3414" t="n">
+        <v>66</v>
+      </c>
+      <c r="D3414" t="n">
+        <v>37</v>
+      </c>
+      <c r="E3414" t="n">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="3415">
+      <c r="A3415" t="n">
+        <v>39</v>
+      </c>
+      <c r="B3415" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3415" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3415" t="n">
+        <v>61</v>
+      </c>
+      <c r="E3415" t="n">
+        <v>558</v>
+      </c>
+    </row>
+    <row r="3416">
+      <c r="A3416" t="n">
+        <v>40</v>
+      </c>
+      <c r="B3416" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3416" t="n">
+        <v>91</v>
+      </c>
+      <c r="D3416" t="n">
+        <v>33</v>
+      </c>
+      <c r="E3416" t="n">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="3417">
+      <c r="A3417" t="n">
+        <v>41</v>
+      </c>
+      <c r="B3417" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3417" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3417" t="n">
+        <v>95</v>
+      </c>
+      <c r="E3417" t="n">
+        <v>559</v>
+      </c>
+    </row>
+    <row r="3418">
+      <c r="A3418" t="n">
+        <v>42</v>
+      </c>
+      <c r="B3418" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3418" t="n">
+        <v>80</v>
+      </c>
+      <c r="D3418" t="n">
+        <v>73</v>
+      </c>
+      <c r="E3418" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3419">
+      <c r="A3419" t="n">
+        <v>43</v>
+      </c>
+      <c r="B3419" t="n">
+        <v>2</v>
+      </c>
+      <c r="C3419" t="n">
+        <v>96</v>
+      </c>
+      <c r="D3419" t="n">
+        <v>87</v>
+      </c>
+      <c r="E3419" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3420">
+      <c r="A3420" t="n">
+        <v>44</v>
+      </c>
+      <c r="B3420" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3420" t="n">
+        <v>18</v>
+      </c>
+      <c r="D3420" t="n">
+        <v>61</v>
+      </c>
+      <c r="E3420" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3421">
+      <c r="A3421" t="n">
+        <v>45</v>
+      </c>
+      <c r="B3421" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3421" t="n">
+        <v>51</v>
+      </c>
+      <c r="D3421" t="n">
+        <v>31</v>
+      </c>
+      <c r="E3421" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3422">
+      <c r="A3422" t="n">
+        <v>46</v>
+      </c>
+      <c r="B3422" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3422" t="n">
+        <v>93</v>
+      </c>
+      <c r="D3422" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3422" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3423">
+      <c r="A3423" t="n">
+        <v>47</v>
+      </c>
+      <c r="B3423" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3423" t="n">
+        <v>78</v>
+      </c>
+      <c r="D3423" t="n">
+        <v>62</v>
+      </c>
+      <c r="E3423" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3424">
+      <c r="A3424" t="n">
+        <v>48</v>
+      </c>
+      <c r="B3424" t="n">
+        <v>7</v>
+      </c>
+      <c r="C3424" t="n">
+        <v>86</v>
+      </c>
+      <c r="D3424" t="n">
+        <v>26</v>
+      </c>
+      <c r="E3424" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3425">
+      <c r="A3425" t="n">
+        <v>49</v>
+      </c>
+      <c r="B3425" t="n">
+        <v>8</v>
+      </c>
+      <c r="C3425" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3425" t="n">
+        <v>89</v>
+      </c>
+      <c r="E3425" t="n">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="3426">
+      <c r="A3426" t="n">
+        <v>50</v>
+      </c>
+      <c r="B3426" t="n">
+        <v>9</v>
+      </c>
+      <c r="C3426" t="n">
+        <v>20</v>
+      </c>
+      <c r="D3426" t="n">
+        <v>63</v>
+      </c>
+      <c r="E3426" t="n">
+        <v>560</v>
       </c>
     </row>
   </sheetData>
@@ -66656,7 +67773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F231"/>
+  <dimension ref="A1:F234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -73105,30 +74222,114 @@
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dbam o Zdrowie Expert </t>
+          <t>Power Kraków</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2182766158</t>
+          <t>7303043147</t>
         </is>
       </c>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Nowy Targ</t>
+          <t>Zakopane</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>Siłownia / klub sportowy</t>
+          <t>Drogeria specjalistyczna</t>
         </is>
       </c>
       <c r="F231" t="n">
-        <v>1</v>
+        <v>15</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="n">
+        <v>242</v>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Pro Muscle Bielsko-Biała</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>8630248238</t>
+        </is>
+      </c>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Gorzów Wielkopolski</t>
+        </is>
+      </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>Sklep internetowy z suplementami</t>
+        </is>
+      </c>
+      <c r="F232" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="n">
+        <v>243</v>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Power Zielona Góra</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>5361536383</t>
+        </is>
+      </c>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Tarnobrzeg</t>
+        </is>
+      </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>Zielarnia</t>
+        </is>
+      </c>
+      <c r="F233" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="n">
+        <v>244</v>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Vita Max</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>7440930474</t>
+        </is>
+      </c>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Cieszyn</t>
+        </is>
+      </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>Sklep internetowy z suplementami</t>
+        </is>
+      </c>
+      <c r="F234" t="n">
+        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>